<commit_message>
Apply manual fixes and updates post upgrade
- Fix ql.BusinessDayConvention conversion
- Remove settlement days input from Excel qlMake... constructors
- Add constructor qlMakeCreditDefaultSwap
  * Note: argument dateGenerationRule is broken in SWIG
- Remove deprecated Kruger interpolated zero curves
- Fix qlBlackVarianceCurve and add Excel example
- Update qlMultipleResetsSwapRateHelper and add unittest
- Add qlMakeSwaption unittest and excel example
- Add FX forward example sheet for new module
</commit_message>
<xml_diff>
--- a/tests/workbooktests/workbooks/test_creditdefaultswap.xlsx
+++ b/tests/workbooktests/workbooks/test_creditdefaultswap.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\tests\workbooktests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47BD23CE-B565-4699-8F63-64E5BC388FAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95DE1F39-3FF2-41EF-898E-C6AD3443869C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3450" yWindow="-18675" windowWidth="30690" windowHeight="16530" xr2:uid="{91D19581-6C36-46DE-A860-F049E5DCF68D}"/>
+    <workbookView xWindow="-120" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{91D19581-6C36-46DE-A860-F049E5DCF68D}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="qlCreditdefaultswap" sheetId="1" r:id="rId1"/>
+    <sheet name="qlMakeCreditDefaultSwap" sheetId="3" r:id="rId2"/>
+    <sheet name="qlCdsOption" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -61,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="108">
   <si>
     <t>Evaluation date</t>
   </si>
@@ -303,16 +305,88 @@
     <t>qlCdsOption</t>
   </si>
   <si>
-    <t>Default curve</t>
-  </si>
-  <si>
-    <t>Discount curve</t>
-  </si>
-  <si>
     <t>Volatility</t>
   </si>
   <si>
     <t>qlBlackCdsOptionEngine</t>
+  </si>
+  <si>
+    <t>NPV</t>
+  </si>
+  <si>
+    <t>maturity</t>
+  </si>
+  <si>
+    <t>The maturity of the CDS (as a qDate or qPeriod).</t>
+  </si>
+  <si>
+    <t>running_spread</t>
+  </si>
+  <si>
+    <t>The running spread of the CDS.</t>
+  </si>
+  <si>
+    <t>upfront_rate</t>
+  </si>
+  <si>
+    <t>The upfront rate of the CDS (optional).</t>
+  </si>
+  <si>
+    <t>side</t>
+  </si>
+  <si>
+    <t>The protection side of the CDS (BUY/SELL) (optional).</t>
+  </si>
+  <si>
+    <t>The notional amount of the CDS (optional).</t>
+  </si>
+  <si>
+    <t>coupon_tenor</t>
+  </si>
+  <si>
+    <t>The coupon tenor of the CDS (as a qPeriod) (optional).</t>
+  </si>
+  <si>
+    <t>The day counter of the CDS (optional).</t>
+  </si>
+  <si>
+    <t>The day counter for the last period of the CDS (optional).</t>
+  </si>
+  <si>
+    <t>date_generation_rule</t>
+  </si>
+  <si>
+    <t>The date generation rule for the CDS (optional).</t>
+  </si>
+  <si>
+    <t>The number of cash settlement days for the CDS (optional).</t>
+  </si>
+  <si>
+    <t>pricing_engine</t>
+  </si>
+  <si>
+    <t>The pricing engine to use for the CDS (optional).</t>
+  </si>
+  <si>
+    <t>The trade date of the CDS (as a qDate) (optional).</t>
+  </si>
+  <si>
+    <t>5Y</t>
+  </si>
+  <si>
+    <t>3m</t>
+  </si>
+  <si>
+    <t>Act/360</t>
+  </si>
+  <si>
+    <t>qlMakeCreditDefaultSwap</t>
+  </si>
+  <si>
+    <t>dateGenerationRule argument is currently broken in SWIG</t>
+  </si>
+  <si>
+    <t>nominal</t>
   </si>
 </sst>
 </file>
@@ -322,7 +396,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -334,6 +408,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -359,7 +440,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -379,6 +460,10 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -715,7 +800,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA12D9BF-7D17-481B-B93D-02FD550C5515}">
-  <dimension ref="A1:H134"/>
+  <dimension ref="A1:V110"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.5546875" bestFit="1" customWidth="1"/>
@@ -735,9 +820,9 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="e" cm="1">
-        <f t="array" aca="1" ref="B2" ca="1">_xll.qlSettingsSetEvaluationDate(B1)</f>
-        <v>#VALUE!</v>
+      <c r="B2" s="5" cm="1">
+        <f t="array" ref="B2">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>46174</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -747,18 +832,18 @@
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="e" cm="1">
-        <f t="array" aca="1" ref="B4" ca="1">_xll.qlFlatForward(B2,0.03)</f>
-        <v>#VALUE!</v>
+      <c r="B4" s="5" t="str" cm="1">
+        <f t="array" ref="B4">_xll.qlFlatForward(B2,0.03)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R4C2YieldTermStructureHandle,A</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B6" ca="1">_xll.qlFaceValueClaim()</f>
-        <v>#VALUE!</v>
+      <c r="B6" s="3" t="str" cm="1">
+        <f t="array" ref="B6">_xll.qlFaceValueClaim()</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R6C2FaceValueClaim,A</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -781,9 +866,9 @@
       <c r="A10" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="5" t="e" cm="1">
-        <f t="array" aca="1" ref="B10" ca="1">_xll.qlCdsMaturity(B2,B8,B9)</f>
-        <v>#VALUE!</v>
+      <c r="B10" s="5" cm="1">
+        <f t="array" ref="B10">_xll.qlCdsMaturity(B2,B8,B9)</f>
+        <v>48019</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -798,9 +883,9 @@
       <c r="A12" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B12" ca="1">_xll.qlMakeSchedule(B11,B10,"3m",,"Ldn","following")</f>
-        <v>#VALUE!</v>
+      <c r="B12" s="3" t="str" cm="1">
+        <f t="array" ref="B12">_xll.qlMakeSchedule(B11,B10,"3m",,"Ldn","following")</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R12C2Schedule,A</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
@@ -815,9 +900,9 @@
       <c r="A15" t="s">
         <v>59</v>
       </c>
-      <c r="B15" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B15" ca="1">_xll.qlFlatHazardRate(B2,0.03,"Act/365")</f>
-        <v>#VALUE!</v>
+      <c r="B15" s="3" t="str" cm="1">
+        <f t="array" ref="B15">_xll.qlFlatHazardRate(B2,0.03,"Act/365")</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R15C2DefaultProbabilityTermStructureHandle,A</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
@@ -871,13 +956,13 @@
       <c r="A21" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="3" t="e">
-        <f ca="1">$B$12</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C21" s="3" t="e">
-        <f ca="1">$B$12</f>
-        <v>#VALUE!</v>
+      <c r="B21" s="3" t="str">
+        <f>$B$12</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R12C2Schedule,A</v>
+      </c>
+      <c r="C21" s="3" t="str">
+        <f>$B$12</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R12C2Schedule,A</v>
       </c>
       <c r="H21" t="s">
         <v>12</v>
@@ -949,9 +1034,9 @@
       <c r="A27" t="s">
         <v>23</v>
       </c>
-      <c r="B27" s="3" t="e">
-        <f ca="1">B6</f>
-        <v>#VALUE!</v>
+      <c r="B27" s="3" t="str">
+        <f>B6</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R6C2FaceValueClaim,A</v>
       </c>
       <c r="H27" t="s">
         <v>24</v>
@@ -995,161 +1080,221 @@
       <c r="A31" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B31" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B31" ca="1">_xll.qlCreditDefaultSwap(B18,B19,B20,B21,B22,B23,B24,B25,B26,B27,B28,B29,B30)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C31" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="C31" ca="1">_xll.qlCreditDefaultSwap(C18,C19,C20,C21,C22,C23)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B31" s="3" t="str" cm="1">
+        <f t="array" ref="B31">_xll.qlCreditDefaultSwap(B18,B19,B20,B21,B22,B23,B24,B25,B26,B27,B28,B29,B30)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R31C2CreditDefaultSwap,A</v>
+      </c>
+      <c r="C31" s="3" t="str" cm="1">
+        <f t="array" ref="C31">_xll.qlCreditDefaultSwap(C18,C19,C20,C21,C22,C23)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R31C3CreditDefaultSwap,A</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>42</v>
       </c>
-      <c r="B33" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B33" ca="1">_xll.qlCreditdefaultswapSide(B31)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B33" s="3" t="str" cm="1">
+        <f t="array" ref="B33">_xll.qlCreditdefaultswapSide(B31)</f>
+        <v>BUY</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>43</v>
       </c>
-      <c r="B34" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B34" ca="1">_xll.qlCreditDefaultSwapNotional(B31)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B34" s="3" cm="1">
+        <f t="array" ref="B34">_xll.qlCreditDefaultSwapNotional(B31)</f>
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>44</v>
       </c>
-      <c r="B35" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B35" ca="1">_xll.qlCreditDefaultSwapRunningSpread(B31)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B35" s="3" cm="1">
+        <f t="array" ref="B35">_xll.qlCreditDefaultSwapRunningSpread(B31)</f>
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>45</v>
       </c>
-      <c r="B36" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B36" ca="1">_xll.qlCreditDefaultSwapUpfront(B31)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B36" s="3" t="str" cm="1">
+        <f t="array" ref="B36">_xll.qlCreditDefaultSwapUpfront(B31)</f>
+        <v>Expected python float, got 'None'</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>46</v>
       </c>
-      <c r="B37" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B37" ca="1">_xll.qlCreditdefaultSwapSettlesAccrual(B31)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B37" s="3" t="b" cm="1">
+        <f t="array" ref="B37">_xll.qlCreditdefaultSwapSettlesAccrual(B31)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>47</v>
       </c>
-      <c r="B38" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B38" ca="1">_xll.qlCreditdefaultswapPaysAtDefaultTime(B31)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B38" s="3" t="b" cm="1">
+        <f t="array" ref="B38">_xll.qlCreditdefaultswapPaysAtDefaultTime(B31)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>48</v>
       </c>
-      <c r="B39" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B39" ca="1">TRANSPOSE(_xll.qlCreditDefaultSwapCoupons(B31))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B39" s="3" t="str" cm="1">
+        <f t="array" ref="B39:V39">TRANSPOSE(_xll.qlCreditDefaultSwapCoupons(B31))</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,A</v>
+      </c>
+      <c r="C39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,B</v>
+      </c>
+      <c r="D39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,C</v>
+      </c>
+      <c r="E39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,D</v>
+      </c>
+      <c r="F39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,E</v>
+      </c>
+      <c r="G39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,F</v>
+      </c>
+      <c r="H39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,G</v>
+      </c>
+      <c r="I39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,H</v>
+      </c>
+      <c r="J39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,I</v>
+      </c>
+      <c r="K39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,J</v>
+      </c>
+      <c r="L39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,K</v>
+      </c>
+      <c r="M39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,L</v>
+      </c>
+      <c r="N39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,M</v>
+      </c>
+      <c r="O39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,N</v>
+      </c>
+      <c r="P39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,O</v>
+      </c>
+      <c r="Q39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,P</v>
+      </c>
+      <c r="R39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,Q</v>
+      </c>
+      <c r="S39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,R</v>
+      </c>
+      <c r="T39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,S</v>
+      </c>
+      <c r="U39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,T</v>
+      </c>
+      <c r="V39" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R39C2CashFlow,U</v>
+      </c>
+    </row>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>49</v>
       </c>
-      <c r="B40" s="5" t="e" cm="1">
-        <f t="array" aca="1" ref="B40" ca="1">_xll.qlCreditDefaultSwapProtectionStartDate(B31)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B40" s="5" cm="1">
+        <f t="array" ref="B40">_xll.qlCreditDefaultSwapProtectionStartDate(B31)</f>
+        <v>46101</v>
+      </c>
+    </row>
+    <row r="41" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>50</v>
       </c>
-      <c r="B41" s="5" t="e" cm="1">
-        <f t="array" aca="1" ref="B41" ca="1">_xll.qlCreditDefaultSwapProtectionEndDate(B31)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B41" s="5" cm="1">
+        <f t="array" ref="B41">_xll.qlCreditDefaultSwapProtectionEndDate(B31)</f>
+        <v>48019</v>
+      </c>
+    </row>
+    <row r="42" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>51</v>
       </c>
-      <c r="B42" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B42" ca="1">_xll.qlCreditDefaultSwapRebatesAccrual(B31)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B42" s="3" t="b" cm="1">
+        <f t="array" ref="B42">_xll.qlCreditDefaultSwapRebatesAccrual(B31)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>52</v>
       </c>
-      <c r="B43" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B43" ca="1">_xll.qlCreditDefaultswapUpfrontPayment(B31)</f>
-        <v>#VALUE!</v>
+      <c r="B43" s="3" t="str" cm="1">
+        <f t="array" ref="B43">_xll.qlCreditDefaultswapUpfrontPayment(B31)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R43C2CashFlow,A</v>
       </c>
       <c r="C43" s="1"/>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>53</v>
       </c>
-      <c r="B44" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B44" ca="1">_xll.qlCreditDefaultSwapAccrualRebate(B31)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B44" s="3" t="str" cm="1">
+        <f t="array" ref="B44">_xll.qlCreditDefaultSwapAccrualRebate(B31)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R44C2CashFlow,A</v>
+      </c>
+    </row>
+    <row r="45" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>54</v>
       </c>
-      <c r="B45" s="5" t="e" cm="1">
-        <f t="array" aca="1" ref="B45" ca="1">_xll.qlCreditDefaultSwapTradeDate(B31)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B45" s="5" cm="1">
+        <f t="array" ref="B45">_xll.qlCreditDefaultSwapTradeDate(B31)</f>
+        <v>46101</v>
+      </c>
+    </row>
+    <row r="46" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>55</v>
       </c>
-      <c r="B46" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B46" ca="1">_xll.qlCreditDefaultSwapCashSettlementDays(B31)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B46" s="3" cm="1">
+        <f t="array" ref="B46">_xll.qlCreditDefaultSwapCashSettlementDays(B31)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:22" x14ac:dyDescent="0.3">
       <c r="B47" s="4"/>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>57</v>
       </c>
-      <c r="B49" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B49" ca="1">_xll.qlCreditDefaultSwapImpliedHazardRate(B31,0,B4,"Act/365",B14)</f>
-        <v>#VALUE!</v>
+      <c r="B49" s="3" cm="1">
+        <f t="array" ref="B49">_xll.qlCreditDefaultSwapImpliedHazardRate(B31,0,B4,"Act/365",B14)</f>
+        <v>5.2957081659976007E-2</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>60</v>
       </c>
-      <c r="B50" s="8" t="e" cm="1">
-        <f t="array" aca="1" ref="B50" ca="1">_xll.qlCreditDefaultSwapConventionalSpread(B31,B14,B4,"Act/365","ISDA")</f>
-        <v>#VALUE!</v>
+      <c r="B50" s="8" cm="1">
+        <f t="array" ref="B50">_xll.qlCreditDefaultSwapConventionalSpread(B31,B14,B4,"Act/365","ISDA")</f>
+        <v>2.9999999996653062E-2</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
@@ -1164,52 +1309,52 @@
       <c r="A53" t="s">
         <v>61</v>
       </c>
-      <c r="B53" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B53" ca="1">_xll.qlMidPointCdsEngine($B$15,$B$14,$B$4)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C53" t="e" cm="1">
-        <f t="array" aca="1" ref="C53" ca="1">_xll.qlInstrumentNPV($B$31,_xll.qlInstrumentSetPricingEngine($B$31,B53))</f>
-        <v>#VALUE!</v>
+      <c r="B53" s="3" t="str" cm="1">
+        <f t="array" ref="B53">_xll.qlMidPointCdsEngine($B$15,$B$14,$B$4)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R53C2MidPointCdsEngine,A</v>
+      </c>
+      <c r="C53" cm="1">
+        <f t="array" ref="C53">_xll.qlInstrumentNPV($B$31,_xll.qlInstrumentSetPricingEngine($B$31,B53))</f>
+        <v>-597.18654960901893</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>62</v>
       </c>
-      <c r="B54" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B54" ca="1">_xll.qlIntegralCdsEngine("1m",$B$15,$B$14,$B$4,FALSE)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C54" t="e" cm="1">
-        <f t="array" aca="1" ref="C54" ca="1">_xll.qlInstrumentNPV($B$31,_xll.qlInstrumentSetPricingEngine($B$31,B54))</f>
-        <v>#VALUE!</v>
+      <c r="B54" s="3" t="str" cm="1">
+        <f t="array" ref="B54">_xll.qlIntegralCdsEngine("1m",$B$15,$B$14,$B$4,FALSE)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R54C2IntegralCdsEngine,A</v>
+      </c>
+      <c r="C54" cm="1">
+        <f t="array" ref="C54">_xll.qlInstrumentNPV($B$31,_xll.qlInstrumentSetPricingEngine($B$31,B54))</f>
+        <v>-599.8333220606329</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>63</v>
       </c>
-      <c r="B55" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B55" ca="1">_xll.qlIsdaCdsEngine($B$15,$B$14,$B$4,FALSE,"Taylor","Half_Day_Bias","Piecewise")</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C55" t="e" cm="1">
-        <f t="array" aca="1" ref="C55" ca="1">_xll.qlInstrumentNPV($B$31,_xll.qlInstrumentSetPricingEngine($B$31,B55))</f>
-        <v>#VALUE!</v>
+      <c r="B55" s="3" t="str" cm="1">
+        <f t="array" ref="B55">_xll.qlIsdaCdsEngine($B$15,$B$14,$B$4,FALSE,"Taylor","Half_Day_Bias","Piecewise")</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R55C2IsdaCdsEngine,A</v>
+      </c>
+      <c r="C55" cm="1">
+        <f t="array" ref="C55">_xll.qlInstrumentNPV($B$31,_xll.qlInstrumentSetPricingEngine($B$31,B55))</f>
+        <v>-597.3783443237852</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>63</v>
       </c>
-      <c r="B56" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B56" ca="1">_xll.qlIsdaCdsEngine($B$15,$B$14,$B$4)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C56" t="e" cm="1">
-        <f t="array" aca="1" ref="C56" ca="1">_xll.qlInstrumentNPV($B$31,_xll.qlInstrumentSetPricingEngine($B$31,B56))</f>
-        <v>#VALUE!</v>
+      <c r="B56" s="3" t="str" cm="1">
+        <f t="array" ref="B56">_xll.qlIsdaCdsEngine($B$15,$B$14,$B$4)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R56C2IsdaCdsEngine,A</v>
+      </c>
+      <c r="C56" cm="1">
+        <f t="array" ref="C56">_xll.qlInstrumentNPV($B$31,_xll.qlInstrumentSetPricingEngine($B$31,B56))</f>
+        <v>-597.3783443237852</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
@@ -1265,13 +1410,13 @@
       <c r="A64" t="s">
         <v>11</v>
       </c>
-      <c r="B64" s="3" t="e">
-        <f ca="1">$B$12</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C64" s="3" t="e">
-        <f ca="1">$B$12</f>
-        <v>#VALUE!</v>
+      <c r="B64" s="3" t="str">
+        <f>$B$12</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R12C2Schedule,A</v>
+      </c>
+      <c r="C64" s="3" t="str">
+        <f>$B$12</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R12C2Schedule,A</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
@@ -1325,18 +1470,18 @@
       <c r="A70" t="s">
         <v>66</v>
       </c>
-      <c r="B70" s="5" t="e">
-        <f ca="1">B2+1</f>
-        <v>#VALUE!</v>
+      <c r="B70" s="5">
+        <f>B2+1</f>
+        <v>46175</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>23</v>
       </c>
-      <c r="B71" s="3" t="e">
-        <f ca="1">B6</f>
-        <v>#VALUE!</v>
+      <c r="B71" s="3" t="str">
+        <f>B6</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R6C2FaceValueClaim,A</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
@@ -1376,160 +1521,220 @@
       <c r="A76" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B76" s="4" t="e" cm="1">
-        <f t="array" aca="1" ref="B76" ca="1">_xll.qlCreditDefaultSwapWithUpfront(B60,B61,B62,B63,B64,B65,B66,B67,B68,B69,B70,B71,B72,B73,B74,B75)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C76" s="4" t="e" cm="1">
-        <f t="array" aca="1" ref="C76" ca="1">_xll.qlCreditDefaultSwapWithUpfront(C60,C61,C62,C63,C64,C65,C66)</f>
-        <v>#VALUE!</v>
+      <c r="B76" s="4" t="str" cm="1">
+        <f t="array" ref="B76">_xll.qlCreditDefaultSwapWithUpfront(B60,B61,B62,B63,B64,B65,B66,B67,B68,B69,B70,B71,B72,B73,B74,B75)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R76C2CreditDefaultSwap,A</v>
+      </c>
+      <c r="C76" s="4" t="str" cm="1">
+        <f t="array" ref="C76">_xll.qlCreditDefaultSwapWithUpfront(C60,C61,C62,C63,C64,C65,C66)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R76C3CreditDefaultSwap,A</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>42</v>
       </c>
-      <c r="B78" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B78" ca="1">_xll.qlCreditdefaultswapSide(B76)</f>
-        <v>#VALUE!</v>
+      <c r="B78" s="3" t="str" cm="1">
+        <f t="array" ref="B78">_xll.qlCreditdefaultswapSide(B76)</f>
+        <v>BUY</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>43</v>
       </c>
-      <c r="B79" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B79" ca="1">_xll.qlCreditDefaultSwapNotional(B76)</f>
-        <v>#VALUE!</v>
+      <c r="B79" s="3" cm="1">
+        <f t="array" ref="B79">_xll.qlCreditDefaultSwapNotional(B76)</f>
+        <v>10000</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>44</v>
       </c>
-      <c r="B80" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B80" ca="1">_xll.qlCreditDefaultSwapRunningSpread(B76)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B80" s="3" cm="1">
+        <f t="array" ref="B80">_xll.qlCreditDefaultSwapRunningSpread(B76)</f>
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="81" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>45</v>
       </c>
-      <c r="B81" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B81" ca="1">_xll.qlCreditDefaultSwapUpfront(B76)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B81" s="3" cm="1">
+        <f t="array" ref="B81">_xll.qlCreditDefaultSwapUpfront(B76)</f>
+        <v>500</v>
+      </c>
+    </row>
+    <row r="82" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>46</v>
       </c>
-      <c r="B82" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B82" ca="1">_xll.qlCreditdefaultSwapSettlesAccrual(B76)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B82" s="3" t="b" cm="1">
+        <f t="array" ref="B82">_xll.qlCreditdefaultSwapSettlesAccrual(B76)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>47</v>
       </c>
-      <c r="B83" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B83" ca="1">_xll.qlCreditdefaultswapPaysAtDefaultTime(B76)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B83" s="3" t="b" cm="1">
+        <f t="array" ref="B83">_xll.qlCreditdefaultswapPaysAtDefaultTime(B76)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>48</v>
       </c>
-      <c r="B84" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B84" ca="1">TRANSPOSE(_xll.qlCreditDefaultSwapCoupons(B76))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B84" s="3" t="str" cm="1">
+        <f t="array" ref="B84:V84">TRANSPOSE(_xll.qlCreditDefaultSwapCoupons(B76))</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,A</v>
+      </c>
+      <c r="C84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,B</v>
+      </c>
+      <c r="D84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,C</v>
+      </c>
+      <c r="E84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,D</v>
+      </c>
+      <c r="F84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,E</v>
+      </c>
+      <c r="G84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,F</v>
+      </c>
+      <c r="H84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,G</v>
+      </c>
+      <c r="I84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,H</v>
+      </c>
+      <c r="J84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,I</v>
+      </c>
+      <c r="K84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,J</v>
+      </c>
+      <c r="L84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,K</v>
+      </c>
+      <c r="M84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,L</v>
+      </c>
+      <c r="N84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,M</v>
+      </c>
+      <c r="O84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,N</v>
+      </c>
+      <c r="P84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,O</v>
+      </c>
+      <c r="Q84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,P</v>
+      </c>
+      <c r="R84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,Q</v>
+      </c>
+      <c r="S84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,R</v>
+      </c>
+      <c r="T84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,S</v>
+      </c>
+      <c r="U84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,T</v>
+      </c>
+      <c r="V84" t="str">
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R84C2CashFlow,U</v>
+      </c>
+    </row>
+    <row r="85" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>49</v>
       </c>
-      <c r="B85" s="5" t="e" cm="1">
-        <f t="array" aca="1" ref="B85" ca="1">_xll.qlCreditDefaultSwapProtectionStartDate(B76)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B85" s="5" cm="1">
+        <f t="array" ref="B85">_xll.qlCreditDefaultSwapProtectionStartDate(B76)</f>
+        <v>46101</v>
+      </c>
+    </row>
+    <row r="86" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>50</v>
       </c>
-      <c r="B86" s="5" t="e" cm="1">
-        <f t="array" aca="1" ref="B86" ca="1">_xll.qlCreditDefaultSwapProtectionEndDate(B76)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B86" s="5" cm="1">
+        <f t="array" ref="B86">_xll.qlCreditDefaultSwapProtectionEndDate(B76)</f>
+        <v>48019</v>
+      </c>
+    </row>
+    <row r="87" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>51</v>
       </c>
-      <c r="B87" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B87" ca="1">_xll.qlCreditDefaultSwapRebatesAccrual(B76)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B87" s="3" t="b" cm="1">
+        <f t="array" ref="B87">_xll.qlCreditDefaultSwapRebatesAccrual(B76)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>52</v>
       </c>
-      <c r="B88" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B88" ca="1">_xll.qlCreditDefaultswapUpfrontPayment(B76)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B88" s="3" t="str" cm="1">
+        <f t="array" ref="B88">_xll.qlCreditDefaultswapUpfrontPayment(B76)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R88C2CashFlow,A</v>
+      </c>
+    </row>
+    <row r="89" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>53</v>
       </c>
-      <c r="B89" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B89" ca="1">_xll.qlCreditDefaultSwapAccrualRebate(B76)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B89" s="3" t="str" cm="1">
+        <f t="array" ref="B89">_xll.qlCreditDefaultSwapAccrualRebate(B76)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R89C2CashFlow,A</v>
+      </c>
+    </row>
+    <row r="90" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>54</v>
       </c>
-      <c r="B90" s="5" t="e" cm="1">
-        <f t="array" aca="1" ref="B90" ca="1">_xll.qlCreditDefaultSwapTradeDate(B76)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B90" s="5" cm="1">
+        <f t="array" ref="B90">_xll.qlCreditDefaultSwapTradeDate(B76)</f>
+        <v>46101</v>
+      </c>
+    </row>
+    <row r="91" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>55</v>
       </c>
-      <c r="B91" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B91" ca="1">_xll.qlCreditDefaultSwapCashSettlementDays(B76)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B91" s="3" cm="1">
+        <f t="array" ref="B91">_xll.qlCreditDefaultSwapCashSettlementDays(B76)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="94" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>57</v>
       </c>
-      <c r="B94" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B94" ca="1">_xll.qlCreditDefaultSwapImpliedHazardRate(B31,0,B4,"Act/365",B14)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B94" s="3" cm="1">
+        <f t="array" ref="B94">_xll.qlCreditDefaultSwapImpliedHazardRate(B31,0,B4,"Act/365",B14)</f>
+        <v>5.2957081659976007E-2</v>
+      </c>
+    </row>
+    <row r="95" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>60</v>
       </c>
-      <c r="B95" s="8" t="e" cm="1">
-        <f t="array" aca="1" ref="B95" ca="1">_xll.qlCreditDefaultSwapConventionalSpread(B31,B14,B4,"Act/365","ISDA")</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B95" s="8" cm="1">
+        <f t="array" ref="B95">_xll.qlCreditDefaultSwapConventionalSpread(B31,B14,B4,"Act/365","ISDA")</f>
+        <v>2.9999999996653062E-2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:22" x14ac:dyDescent="0.3">
       <c r="B96" s="8"/>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.3">
@@ -1541,276 +1746,550 @@
       <c r="A98" t="s">
         <v>61</v>
       </c>
-      <c r="B98" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B98" ca="1">_xll.qlMidPointCdsEngine($B$15,$B$14,$B$4)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C98" t="e" cm="1">
-        <f t="array" aca="1" ref="C98" ca="1">_xll.qlInstrumentNPV($B$76,_xll.qlInstrumentSetPricingEngine($B$76,B98))</f>
-        <v>#VALUE!</v>
+      <c r="B98" s="3" t="str" cm="1">
+        <f t="array" ref="B98">_xll.qlMidPointCdsEngine($B$15,$B$14,$B$4)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R98C2MidPointCdsEngine,A</v>
+      </c>
+      <c r="C98" cm="1">
+        <f t="array" ref="C98">_xll.qlInstrumentNPV($B$76,_xll.qlInstrumentSetPricingEngine($B$76,B98))</f>
+        <v>-5000185.411268915</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>62</v>
       </c>
-      <c r="B99" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B99" ca="1">_xll.qlIntegralCdsEngine("1m",$B$15,$B$14,$B$4,FALSE)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C99" t="e" cm="1">
-        <f t="array" aca="1" ref="C99" ca="1">_xll.qlInstrumentNPV($B$76,_xll.qlInstrumentSetPricingEngine($B$76,B99))</f>
-        <v>#VALUE!</v>
+      <c r="B99" s="3" t="str" cm="1">
+        <f t="array" ref="B99">_xll.qlIntegralCdsEngine("1m",$B$15,$B$14,$B$4,FALSE)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R99C2IntegralCdsEngine,A</v>
+      </c>
+      <c r="C99" cm="1">
+        <f t="array" ref="C99">_xll.qlInstrumentNPV($B$76,_xll.qlInstrumentSetPricingEngine($B$76,B99))</f>
+        <v>-5000188.0580413667</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>63</v>
       </c>
-      <c r="B100" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B100" ca="1">_xll.qlIsdaCdsEngine($B$15,$B$14,$B$4,FALSE,"Taylor","Half_Day_Bias","Piecewise")</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C100" t="e" cm="1">
-        <f t="array" aca="1" ref="C100" ca="1">_xll.qlInstrumentNPV($B$76,_xll.qlInstrumentSetPricingEngine($B$76,B100))</f>
-        <v>#VALUE!</v>
+      <c r="B100" s="3" t="str" cm="1">
+        <f t="array" ref="B100">_xll.qlIsdaCdsEngine($B$15,$B$14,$B$4,FALSE,"Taylor","Half_Day_Bias","Piecewise")</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R100C2IsdaCdsEngine,A</v>
+      </c>
+      <c r="C100" cm="1">
+        <f t="array" ref="C100">_xll.qlInstrumentNPV($B$76,_xll.qlInstrumentSetPricingEngine($B$76,B100))</f>
+        <v>-5000185.6030636299</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>63</v>
       </c>
-      <c r="B101" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B101" ca="1">_xll.qlIsdaCdsEngine($B$15,$B$14,$B$4)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C101" t="e" cm="1">
-        <f t="array" aca="1" ref="C101" ca="1">_xll.qlInstrumentNPV($B$76,_xll.qlInstrumentSetPricingEngine($B$76,B101))</f>
-        <v>#VALUE!</v>
+      <c r="B101" s="3" t="str" cm="1">
+        <f t="array" ref="B101">_xll.qlIsdaCdsEngine($B$15,$B$14,$B$4)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCreditdefaultswap!R101C2IsdaCdsEngine,A</v>
+      </c>
+      <c r="C101" cm="1">
+        <f t="array" ref="C101">_xll.qlInstrumentNPV($B$76,_xll.qlInstrumentSetPricingEngine($B$76,B101))</f>
+        <v>-5000185.6030636299</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>56</v>
       </c>
-      <c r="B103" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B103" ca="1">_xll.qlCreditDefaultSwapFairUpfront(B76,C98)</f>
-        <v>#VALUE!</v>
+      <c r="B103" s="3" cm="1">
+        <f t="array" ref="B103">_xll.qlCreditDefaultSwapFairUpfront(B76,C98)</f>
+        <v>-5.9904929212237425E-2</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>68</v>
       </c>
-      <c r="B104" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B104" ca="1">_xll.qlCreditDefaultSwapFairSpread(B76,C98)</f>
-        <v>#VALUE!</v>
+      <c r="B104" s="3" cm="1">
+        <f t="array" ref="B104">_xll.qlCreditDefaultSwapFairSpread(B76,C98)</f>
+        <v>1.7005229253407153E-2</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>69</v>
       </c>
-      <c r="B105" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B105" ca="1">_xll.qlCreditDefaultSwapCouponLegBPS(B76,C98)</f>
-        <v>#VALUE!</v>
+      <c r="B105" s="3" cm="1">
+        <f t="array" ref="B105">_xll.qlCreditDefaultSwapCouponLegBPS(B76,C98)</f>
+        <v>-4.61232448876906</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>70</v>
       </c>
-      <c r="B106" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B106" ca="1">_xll.qlCreditDefaultSwapUpfrontBPS(B76,C98)</f>
-        <v>#VALUE!</v>
+      <c r="B106" s="3" cm="1">
+        <f t="array" ref="B106">_xll.qlCreditDefaultSwapUpfrontBPS(B76,C98)</f>
+        <v>-0.99991781159682991</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>71</v>
       </c>
-      <c r="B107" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B107" ca="1">_xll.qlCreditDefaultSwapCouponLegNPV(B76,C98)</f>
-        <v>#VALUE!</v>
+      <c r="B107" s="3" cm="1">
+        <f t="array" ref="B107">_xll.qlCreditDefaultSwapCouponLegNPV(B76,C98)</f>
+        <v>-1383.6973466307179</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>72</v>
       </c>
-      <c r="B108" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B108" ca="1">_xll.qlCreditDefaultSwapDefaultLegNPV(B76,C98)</f>
-        <v>#VALUE!</v>
+      <c r="B108" s="3" cm="1">
+        <f t="array" ref="B108">_xll.qlCreditDefaultSwapDefaultLegNPV(B76,C98)</f>
+        <v>783.86402457008501</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>73</v>
       </c>
-      <c r="B109" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B109" ca="1">_xll.qlCreditDefaultSwapUpfrontNPV(B76,C98)</f>
-        <v>#VALUE!</v>
+      <c r="B109" s="3" cm="1">
+        <f t="array" ref="B109">_xll.qlCreditDefaultSwapUpfrontNPV(B76,C98)</f>
+        <v>-4999589.0579841491</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>74</v>
       </c>
-      <c r="B110" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B110" ca="1">_xll.qlCreditDefaultSwapAccrualRebateNPV(B76,C98)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A113" t="s">
+      <c r="B110" s="3" cm="1">
+        <f t="array" ref="B110">_xll.qlCreditDefaultSwapAccrualRebateNPV(B76,C98)</f>
+        <v>0.83326484299837666</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B91A7F3C-191C-4969-ACFD-5160A0B4D1FE}">
+  <dimension ref="A1:F26"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="33.44140625" customWidth="1"/>
+    <col min="2" max="2" width="74.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="52.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" cm="1">
+        <f t="array" ref="B2">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B3" s="5"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="str" cm="1">
+        <f t="array" ref="B4">_xll.qlFlatForward(B2,0.03)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlMakeCreditDefaultSwap!R4C2YieldTermStructureHandle,A</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="3">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" s="3" t="str" cm="1">
+        <f t="array" ref="B6">_xll.qlFlatHazardRate(B2,0.03,"Act/365")</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlMakeCreditDefaultSwap!R6C2DefaultProbabilityTermStructureHandle,A</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" s="3" t="str" cm="1">
+        <f t="array" ref="B7">_xll.qlMidPointCdsEngine(B6,B5,B4,B2)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlMakeCreditDefaultSwap!R7C2MidPointCdsEngine,A</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="D10" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>87</v>
+      </c>
+      <c r="B11" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="D11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>89</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="B13" s="3">
+        <v>1000</v>
+      </c>
+      <c r="D13" t="s">
+        <v>91</v>
+      </c>
+      <c r="F13" s="9"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>92</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="D14" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D15" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D16" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>96</v>
+      </c>
+      <c r="D17" t="s">
+        <v>97</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>67</v>
+      </c>
+      <c r="B18" s="3">
+        <v>0</v>
+      </c>
+      <c r="D18" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>99</v>
+      </c>
+      <c r="B19" s="3" t="str">
+        <f>B7</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlMakeCreditDefaultSwap!R7C2MidPointCdsEngine,A</v>
+      </c>
+      <c r="D19" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" s="5">
+        <f>B2-10</f>
+        <v>46164</v>
+      </c>
+      <c r="D20" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B21" s="3" t="str" cm="1">
+        <f t="array" ref="B21">_xll.qlMakeCreditDefaultSwap(B9,B10,B11,B12,B13,B14,B15,B16,B17,B18,B19,B20,B2)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlMakeCreditDefaultSwap!R21C2CreditDefaultSwap,A</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>82</v>
+      </c>
+      <c r="B23" s="3" cm="1">
+        <f t="array" ref="B23">_xll.qlInstrumentNPV(B21)</f>
+        <v>32.4172313482213</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" s="3" cm="1">
+        <f t="array" ref="B25">_xll.qlCreditDefaultSwapNotional(B21)</f>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B26" s="10"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68E70A4B-4753-416F-B368-A39CFAB8817E}">
+  <dimension ref="A1:B29"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27.21875" customWidth="1"/>
+    <col min="2" max="2" width="81.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" cm="1">
+        <f t="array" ref="B2">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>75</v>
       </c>
-      <c r="B113" s="5" t="e" cm="1">
-        <f t="array" aca="1" ref="B113" ca="1">_xll.qlCdsMaturity(B2,"1y","CDS")</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A114" t="s">
+      <c r="B4" s="5" cm="1">
+        <f t="array" ref="B4">_xll.qlCdsMaturity(qlCreditdefaultswap!B2,"1y","CDS")</f>
+        <v>46558</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>76</v>
       </c>
-      <c r="B114" s="5" t="e" cm="1">
-        <f t="array" aca="1" ref="B114" ca="1">_xll.qlCdsMaturity(B2,"6y","cds")</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A115" t="s">
+      <c r="B5" s="5" cm="1">
+        <f t="array" ref="B5">_xll.qlCdsMaturity(qlCreditdefaultswap!B2,"6y","cds")</f>
+        <v>48385</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>39</v>
       </c>
-      <c r="B115" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B115" ca="1">_xll.qlMakeSchedule(B113,B114,"3m",,"Ldn","following",,"CDS")</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A116" t="s">
+      <c r="B6" s="3" t="str" cm="1">
+        <f t="array" ref="B6">_xll.qlMakeSchedule(B4,B5,"3m",,"Ldn","following",,"CDS")</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCdsOption!R6C2Schedule,A</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>4</v>
       </c>
-      <c r="B116" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B116" ca="1">_xll.qlCreditDefaultSwap("Buy",10000,0.01,B115,"Following","Actual/360")</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A118" t="s">
+      <c r="B7" s="3" t="str" cm="1">
+        <f t="array" ref="B7">_xll.qlCreditDefaultSwap("Buy",10000,0.01,B6,"Following","Actual/360")</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCdsOption!R7C2CreditDefaultSwap,A</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B8" s="3"/>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>77</v>
       </c>
-      <c r="B118" s="5" t="e" cm="1">
-        <f t="array" aca="1" ref="B118" ca="1">_xll.qlCalendarAdvance2("Ldn",B113,"-2d")</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A119" t="s">
+      <c r="B9" s="5" cm="1">
+        <f t="array" ref="B9">_xll.qlCalendarAdvance2("Ldn",B4,"-2d")</f>
+        <v>46555</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>78</v>
       </c>
-      <c r="B119" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B119" ca="1">_xll.qlEuropeanExercise(B118)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A121" s="6" t="s">
+      <c r="B10" s="3" t="str" cm="1">
+        <f t="array" ref="B10">_xll.qlEuropeanExercise(B9)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCdsOption!R10C2EuropeanExercise,A</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B121" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B121" ca="1">_xll.qlCdsOption(B116,B119)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A122" s="6" t="s">
+      <c r="B12" s="3" t="str" cm="1">
+        <f t="array" ref="B12">_xll.qlCdsOption(B7,B10)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCdsOption!R12C2CdsOption,A</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B122" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B122" ca="1">_xll.qlCdsOption(B116,B119,FALSE)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A124" t="s">
+      <c r="B13" s="3" t="str" cm="1">
+        <f t="array" ref="B13">_xll.qlCdsOption(B7,B10,FALSE)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCdsOption!R13C2CdsOption,A</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="5" t="str" cm="1">
+        <f t="array" ref="B15">_xll.qlFlatForward(B2,0.03)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCdsOption!R15C2YieldTermStructureHandle,A</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>58</v>
+      </c>
+      <c r="B17" s="3">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" s="3" t="str" cm="1">
+        <f t="array" ref="B18">_xll.qlFlatHazardRate(B2,0.03,"Act/365")</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCdsOption!R18C2DefaultProbabilityTermStructureHandle,A</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" s="3" t="str" cm="1">
+        <f t="array" ref="B20">_xll.qlMidPointCdsEngine(B18,B17,B15,B2)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCdsOption!R20C2MidPointCdsEngine,A</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B21" s="3" t="b" cm="1">
+        <f t="array" ref="B21">_xll.qlInstrumentSetPricingEngine(B7,B20,B2)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
         <v>80</v>
       </c>
-      <c r="B124" s="3" t="e">
-        <f ca="1">B15</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A125" t="s">
-        <v>58</v>
-      </c>
-      <c r="B125" s="3">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A126" t="s">
+      <c r="B23" s="3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B126" s="5" t="e">
-        <f ca="1">B4</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A127" t="s">
+      <c r="B25" s="3" t="str" cm="1">
+        <f t="array" ref="B25">_xll.qlBlackCdsOptionEngine(B18,B17,B15,B23,B2)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCdsOption!R25C2BlackCdsOptionEngine,A</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B26" s="3" t="str" cm="1">
+        <f t="array" ref="B26">_xll.qlBlackCdsOptionEngine(B18,B17,B15,B23,B2)</f>
+        <v>欣[test_creditdefaultswap.xlsx]qlCdsOption!R26C2BlackCdsOptionEngine,A</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>82</v>
       </c>
-      <c r="B127" s="3">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A129" t="s">
-        <v>61</v>
-      </c>
-      <c r="B129" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B129" ca="1">_xll.qlMidPointCdsEngine(B124,B125,B126)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B130" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B130" ca="1">_xll.qlInstrumentSetPricingEngine(B116,B129)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C132" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A133" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="B133" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B133" ca="1">_xll.qlBlackCdsOptionEngine(B124,B125,B126,B127,B130)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C133" t="e" cm="1">
-        <f t="array" aca="1" ref="C133" ca="1">_xll.qlInstrumentNPV(B121,_xll.qlInstrumentSetPricingEngine(B121,B133))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A134" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="B134" s="3" t="e" cm="1">
-        <f t="array" aca="1" ref="B134" ca="1">_xll.qlBlackCdsOptionEngine(B124,B125,B126,B127,B130)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C134" t="e" cm="1">
-        <f t="array" aca="1" ref="C134" ca="1">_xll.qlInstrumentNPV(B122,_xll.qlInstrumentSetPricingEngine(B122,B134))</f>
-        <v>#VALUE!</v>
+      <c r="B28" cm="1">
+        <f t="array" ref="B28">_xll.qlInstrumentNPV(B12,_xll.qlInstrumentSetPricingEngine(B12,B25))</f>
+        <v>358.19239828252648</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>82</v>
+      </c>
+      <c r="B29" cm="1">
+        <f t="array" ref="B29">_xll.qlInstrumentNPV(B13,_xll.qlInstrumentSetPricingEngine(B13,B26))</f>
+        <v>537.46850787665062</v>
       </c>
     </row>
   </sheetData>

</xml_diff>